<commit_message>
Capstone-Projekt: TFT-Ergebnisse, Vergleichsplots und Jahresprognose-Notebooks ergänzt.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Capstone Projekt/Benchmark_PM25_Beijing.xlsx
+++ b/Capstone Projekt/Benchmark_PM25_Beijing.xlsx
@@ -8,26 +8,123 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaiws\Claude\Projects\Business Prognosis\capstone projekt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC11CA1-C41C-48A1-9860-82D7FF9000D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_08409C9D4FA301D60256E2A3180D1C8CF3931A9F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Unser Ansatz " sheetId="1" r:id="rId1"/>
-    <sheet name="Literatur (Paper)" sheetId="2" r:id="rId2"/>
-    <sheet name="Datenpaper (Learnings)" sheetId="3" r:id="rId3"/>
-    <sheet name="Hinweise" sheetId="4" r:id="rId4"/>
-    <sheet name="Quellen" sheetId="5" r:id="rId5"/>
+    <sheet name="Zusammenfassung" sheetId="1" r:id="rId1"/>
+    <sheet name="Unser Ansatz " sheetId="2" r:id="rId2"/>
+    <sheet name="TFT (Auswertung)" sheetId="3" r:id="rId3"/>
+    <sheet name="Literatur (Paper)" sheetId="4" r:id="rId4"/>
+    <sheet name="Datenpaper (Learnings)" sheetId="5" r:id="rId5"/>
+    <sheet name="Hinweise" sheetId="6" r:id="rId6"/>
+    <sheet name="Quellen" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Literatur (Paper)'!$A$4:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Literatur (Paper)'!$A$4:$I$20</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="215">
+  <si>
+    <t>Zusammenfassung – beste vergleichbare Modelle (12 Stationen, rollierend, MASE)</t>
+  </si>
+  <si>
+    <t>MASE je Horizont (kleiner = besser; &lt; 1 schlägt naive). Gleicher Split, gleiche rollierende Auswertung. Grün = bestes Modell je Horizont. Getrennt nach Prognose-Setting.</t>
+  </si>
+  <si>
+    <t>A) Perfect Prognosis</t>
+  </si>
+  <si>
+    <t>(Zukunftswetter bekannt – Obergrenze)</t>
+  </si>
+  <si>
+    <t>Modell</t>
+  </si>
+  <si>
+    <t>8 h</t>
+  </si>
+  <si>
+    <t>24 h</t>
+  </si>
+  <si>
+    <t>48 h</t>
+  </si>
+  <si>
+    <t>72 h</t>
+  </si>
+  <si>
+    <t>Prophet + Wetter (Perfect Prognosis)</t>
+  </si>
+  <si>
+    <t>TFT: Basis (univariat, ohne Exog.)</t>
+  </si>
+  <si>
+    <t>TFT: Behandelt + FT + Reg</t>
+  </si>
+  <si>
+    <t>→ bestes Modell</t>
+  </si>
+  <si>
+    <t>TFT
+(0.389)</t>
+  </si>
+  <si>
+    <t>TFT
+(0.480)</t>
+  </si>
+  <si>
+    <t>TFT
+(0.562)</t>
+  </si>
+  <si>
+    <t>TFT
+(0.594)</t>
+  </si>
+  <si>
+    <t>B) Realistisch (Lag)</t>
+  </si>
+  <si>
+    <t>(kein Zukunftswetter – operativ realistisch)</t>
+  </si>
+  <si>
+    <t>Seasonal Naive (Baseline)</t>
+  </si>
+  <si>
+    <t>Prophet + Wetter (Lag)</t>
+  </si>
+  <si>
+    <t>Prophet + Wetter+Co (Lag)</t>
+  </si>
+  <si>
+    <t>TFT Lag: Wetter</t>
+  </si>
+  <si>
+    <t>TFT Lag: Wetter+Co</t>
+  </si>
+  <si>
+    <t>TFT Lag
+(0.498)</t>
+  </si>
+  <si>
+    <t>TFT Lag
+(0.677)</t>
+  </si>
+  <si>
+    <t>TFT Lag
+(0.872)</t>
+  </si>
+  <si>
+    <t>TFT Lag
+(0.945)</t>
+  </si>
+  <si>
+    <t>Fazit: TFT gewinnt in BEIDEN Settings jeden Horizont. Realistisch (ohne Zukunftswetter) ist TFT Lag: Wetter das beste Modell (0,50/0,68/0,87/0,95) und bleibt als einziges auf allen Horizonten unter 1. Prophet+Co ist nur kurzfristig (8 h) konkurrenzfähig, fällt ab 48 h aber über die naive Baseline. Kennt man das Zukunftswetter (Perfect Prognosis), zieht TFT weiter davon (72 h: 0,59). Kurz: TFT ist robuster über den Horizont und der klare Sieger.</t>
+  </si>
   <si>
     <t>Unser Ansatz – PM2.5-Vorhersage nach Horizont (Einzelstart 1.3.2016)</t>
   </si>
@@ -116,24 +213,87 @@
     <t>D) Rollierend, alle 12 Stationen — Co-Schadstoffe als LAG (Durchschnitts-Startpunkt): Wetter vs. Wetter+Co</t>
   </si>
   <si>
-    <t>Prophet + Wetter (Lag)</t>
-  </si>
-  <si>
-    <t>Prophet + Wetter+Co (Lag)</t>
-  </si>
-  <si>
     <t>Repräsentativ (Mittel über Stationen &amp; Startpunkte): Co-Schadstoffe als Lag senken den 8-h-MASE von 1,02 auf 0,57 und schlagen die Baseline bis ~48 h — leakage-frei.</t>
   </si>
   <si>
+    <t>TFT (Temporal Fusion Transformer) – Auswertung, vergleichbar zu Prophet</t>
+  </si>
+  <si>
+    <t>Rollierende 72-h-Fenster über das Testjahr, nach Lead-Zeit gebucketet (wie Prophet 12.3). MASE &lt; 1 = besser als naive Baseline.</t>
+  </si>
+  <si>
+    <t>— Perfect Prognosis (echtes Zukunftswetter bekannt) —</t>
+  </si>
+  <si>
+    <t>A) Detailstation Aotizhongxin</t>
+  </si>
+  <si>
+    <t>TFT: Basis (univariat)</t>
+  </si>
+  <si>
+    <t>B) Alle 12 Stationen (globales TFT)</t>
+  </si>
+  <si>
+    <t>TFT 12 Stat.: Basis (univariat)</t>
+  </si>
+  <si>
+    <t>TFT 12 Stat.: Behandelt + FT + Reg</t>
+  </si>
+  <si>
+    <t>— Realistisch: Lag (Wetter/Co nur historisch, KEIN Zukunftswetter) —</t>
+  </si>
+  <si>
+    <t>C) Detailstation Aotizhongxin (Lag)</t>
+  </si>
+  <si>
+    <t>D) Alle 12 Stationen (globales TFT, Lag)</t>
+  </si>
+  <si>
+    <t>TFT 12 Stat. Lag: Wetter</t>
+  </si>
+  <si>
+    <t>TFT 12 Stat. Lag: Wetter+Co</t>
+  </si>
+  <si>
+    <t>Interpretation</t>
+  </si>
+  <si>
+    <t>Kernbefund</t>
+  </si>
+  <si>
+    <t>TFT ist in BEIDEN Settings das stärkste Modell und schlägt Prophet auf allen Horizonten. Perfect-Prognosis (12 Stat.): MASE 0,44/0,48/0,56/0,59. Realistisch/Lag (12 Stat.): 0,50/0,68/0,87/0,95 — bleibt überall &lt; 1 (besser als naive).</t>
+  </si>
+  <si>
+    <t>Zukunftswetter zählt</t>
+  </si>
+  <si>
+    <t>Der Sprung von Lag zu Perfect Prognosis ist bei langen Horizonten groß (72 h: 0,95 → 0,59). Zukünftiges Wetter ist für 2–3-Tage-Prognosen sehr informativ.</t>
+  </si>
+  <si>
+    <t>Stabilität</t>
+  </si>
+  <si>
+    <t>Prophet+Co (Lag) startet gut (8 h 0,57), zerfällt aber (72 h 1,11 &gt; naive). TFT-Lag bleibt flach (0,50 → 0,95). Der Temporal-Fusion-Decoder hält längere Horizonte.</t>
+  </si>
+  <si>
+    <t>Co-Schadstoffe</t>
+  </si>
+  <si>
+    <t>Als Lag-Faktor helfen Co-Schadstoffe bei TFT nur minimal und uneinheitlich (Einzelstation leicht besser, 12 Stat. leicht schlechter bei 72 h). Anders als bei Prophet, wo Co den Kurzhorizont stark hebt.</t>
+  </si>
+  <si>
+    <t>Caveats</t>
+  </si>
+  <si>
+    <t>Globales 12-Stationen-Modell (Cross-Station-Lernen) vs. Prophets 12 Einzelmodelle; nur MAX_STEPS=1000 (mehr Training → eher noch besser).</t>
+  </si>
+  <si>
     <t>Andere Modelle auf dem (gleichen / einem) Beijing-Datensatz</t>
   </si>
   <si>
     <t>Grün = echtes h-voraus-Forecasting (direkt vergleichbar). Rest meist NOWCASTING (gleiche Stunde). Siehe 'Hinweise'.</t>
   </si>
   <si>
-    <t>Modell</t>
-  </si>
-  <si>
     <t>Modelltyp</t>
   </si>
   <si>
@@ -518,10 +678,10 @@
     <t>UCI ML Repository #501 – https://archive.ics.uci.edu/dataset/501/beijing+multi+site+air+quality+data</t>
   </si>
   <si>
+    <t>Eure Ergebnisse</t>
+  </si>
+  <si>
     <t>Notebook 03, Abschnitte 8/12.1/12.2/12.3 (CSV-Export)</t>
-  </si>
-  <si>
-    <t>Unsere Ergebnisse</t>
   </si>
 </sst>
 </file>
@@ -532,7 +692,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -631,8 +791,48 @@
       <color rgb="FFC4471C"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FF1C3A44"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1C3A44"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1C7293"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1C3A44"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFC4471C"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF666666"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -682,6 +882,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD8EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E7B8"/>
       </patternFill>
     </fill>
   </fills>
@@ -739,7 +949,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -840,13 +1050,38 @@
     <xf numFmtId="165" fontId="5" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="19" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -1150,6 +1385,308 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="5" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="53" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="52"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="33" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="36" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="38">
+        <v>0.95799999999999996</v>
+      </c>
+      <c r="C6" s="38">
+        <v>0.97499999999999998</v>
+      </c>
+      <c r="D6" s="38">
+        <v>0.86699999999999999</v>
+      </c>
+      <c r="E6" s="38">
+        <v>0.79500000000000004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="42">
+        <v>0.38900000000000001</v>
+      </c>
+      <c r="C7" s="38">
+        <v>0.61699999999999999</v>
+      </c>
+      <c r="D7" s="38">
+        <v>0.82399999999999995</v>
+      </c>
+      <c r="E7" s="38">
+        <v>0.89100000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="36" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="38">
+        <v>0.44400000000000001</v>
+      </c>
+      <c r="C8" s="42">
+        <v>0.48</v>
+      </c>
+      <c r="D8" s="42">
+        <v>0.56200000000000006</v>
+      </c>
+      <c r="E8" s="42">
+        <v>0.59399999999999997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="34" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="48" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="48" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="48" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="48" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="52"/>
+      <c r="D11" s="52"/>
+      <c r="E11" s="52"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="38">
+        <v>1.1319999999999999</v>
+      </c>
+      <c r="C13" s="38">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="D13" s="38">
+        <v>1.1679999999999999</v>
+      </c>
+      <c r="E13" s="38">
+        <v>1.127</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="38">
+        <v>1.022</v>
+      </c>
+      <c r="C14" s="38">
+        <v>1.1990000000000001</v>
+      </c>
+      <c r="D14" s="38">
+        <v>1.1619999999999999</v>
+      </c>
+      <c r="E14" s="38">
+        <v>1.0880000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="36" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="38">
+        <v>0.56899999999999995</v>
+      </c>
+      <c r="C15" s="38">
+        <v>0.84599999999999997</v>
+      </c>
+      <c r="D15" s="38">
+        <v>1.0229999999999999</v>
+      </c>
+      <c r="E15" s="38">
+        <v>1.1140000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="42">
+        <v>0.498</v>
+      </c>
+      <c r="C16" s="42">
+        <v>0.67700000000000005</v>
+      </c>
+      <c r="D16" s="42">
+        <v>0.872</v>
+      </c>
+      <c r="E16" s="42">
+        <v>0.94499999999999995</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="36" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="38">
+        <v>0.503</v>
+      </c>
+      <c r="C17" s="38">
+        <v>0.70199999999999996</v>
+      </c>
+      <c r="D17" s="38">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="E17" s="38">
+        <v>1.006</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="34" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="48" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" s="48" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="54" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="52"/>
+      <c r="C20" s="52"/>
+      <c r="D20" s="52"/>
+      <c r="E20" s="52"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="52"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="52"/>
+      <c r="D21" s="52"/>
+      <c r="E21" s="52"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="52"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="52"/>
+      <c r="D22" s="52"/>
+      <c r="E22" s="52"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="52"/>
+      <c r="B23" s="52"/>
+      <c r="C23" s="52"/>
+      <c r="D23" s="52"/>
+      <c r="E23" s="52"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="52"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="52"/>
+      <c r="D24" s="52"/>
+      <c r="E24" s="52"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A20:E24"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B11:E11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1157,45 +1694,45 @@
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="58.54296875" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="42" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
+      <c r="A1" s="56" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -1205,7 +1742,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B6" s="7">
         <v>86.75</v>
@@ -1222,7 +1759,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B7" s="7">
         <v>92.5</v>
@@ -1239,7 +1776,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B8" s="7">
         <v>114.896</v>
@@ -1256,7 +1793,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B9" s="7">
         <v>166.76400000000001</v>
@@ -1273,7 +1810,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B10" s="7">
         <v>63.585999999999999</v>
@@ -1290,7 +1827,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1300,7 +1837,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B12" s="10">
         <v>10.375</v>
@@ -1317,7 +1854,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B13" s="10">
         <v>22.465</v>
@@ -1334,7 +1871,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B14" s="10">
         <v>33.31</v>
@@ -1351,7 +1888,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B15" s="10">
         <v>54.302999999999997</v>
@@ -1368,7 +1905,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B16" s="10">
         <v>40.292999999999999</v>
@@ -1385,7 +1922,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1395,7 +1932,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="12" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B18" s="13">
         <v>37.722000000000001</v>
@@ -1412,7 +1949,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="12" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B19" s="13">
         <v>61.936999999999998</v>
@@ -1429,7 +1966,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="12" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B20" s="13">
         <v>86.201999999999998</v>
@@ -1446,7 +1983,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B21" s="13">
         <v>137.834</v>
@@ -1463,7 +2000,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="12" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B22" s="13">
         <v>74.051000000000002</v>
@@ -1479,51 +2016,51 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="42" t="s">
-        <v>15</v>
-      </c>
-      <c r="B24" s="43"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
+      <c r="A24" s="56" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" s="52"/>
+      <c r="C24" s="52"/>
+      <c r="D24" s="52"/>
+      <c r="E24" s="52"/>
+      <c r="F24" s="52"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="B25" s="43"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
+      <c r="A25" s="58" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="52"/>
+      <c r="C25" s="52"/>
+      <c r="D25" s="52"/>
+      <c r="E25" s="52"/>
+      <c r="F25" s="52"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="F28" s="3"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -1533,7 +2070,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B30" s="7">
         <v>66.841999999999999</v>
@@ -1550,7 +2087,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B31" s="7">
         <v>66.947000000000003</v>
@@ -1567,7 +2104,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="6" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B32" s="7">
         <v>68.572999999999993</v>
@@ -1584,7 +2121,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B33" s="7">
         <v>66.213999999999999</v>
@@ -1601,7 +2138,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -1611,7 +2148,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="9" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B35" s="10">
         <v>56.206000000000003</v>
@@ -1628,7 +2165,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="9" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B36" s="10">
         <v>57.064</v>
@@ -1645,7 +2182,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="9" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B37" s="10">
         <v>50.798000000000002</v>
@@ -1662,7 +2199,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="9" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B38" s="10">
         <v>46.591999999999999</v>
@@ -1679,7 +2216,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -1689,7 +2226,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="12" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B40" s="13">
         <v>60.097000000000001</v>
@@ -1706,7 +2243,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="12" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B41" s="13">
         <v>70.33</v>
@@ -1723,7 +2260,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="12" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B42" s="13">
         <v>68.334999999999994</v>
@@ -1740,7 +2277,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="12" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B43" s="13">
         <v>64.048000000000002</v>
@@ -1756,65 +2293,65 @@
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45" s="44" t="s">
-        <v>21</v>
-      </c>
-      <c r="B45" s="43"/>
-      <c r="C45" s="43"/>
-      <c r="D45" s="43"/>
-      <c r="E45" s="43"/>
-      <c r="F45" s="43"/>
+      <c r="A45" s="57" t="s">
+        <v>50</v>
+      </c>
+      <c r="B45" s="52"/>
+      <c r="C45" s="52"/>
+      <c r="D45" s="52"/>
+      <c r="E45" s="52"/>
+      <c r="F45" s="52"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A46" s="43"/>
-      <c r="B46" s="43"/>
-      <c r="C46" s="43"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="43"/>
-      <c r="F46" s="43"/>
+      <c r="A46" s="52"/>
+      <c r="B46" s="52"/>
+      <c r="C46" s="52"/>
+      <c r="D46" s="52"/>
+      <c r="E46" s="52"/>
+      <c r="F46" s="52"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A47" s="43"/>
-      <c r="B47" s="43"/>
-      <c r="C47" s="43"/>
-      <c r="D47" s="43"/>
-      <c r="E47" s="43"/>
-      <c r="F47" s="43"/>
+      <c r="A47" s="52"/>
+      <c r="B47" s="52"/>
+      <c r="C47" s="52"/>
+      <c r="D47" s="52"/>
+      <c r="E47" s="52"/>
+      <c r="F47" s="52"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A48" s="43"/>
-      <c r="B48" s="43"/>
-      <c r="C48" s="43"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
+      <c r="A48" s="52"/>
+      <c r="B48" s="52"/>
+      <c r="C48" s="52"/>
+      <c r="D48" s="52"/>
+      <c r="E48" s="52"/>
+      <c r="F48" s="52"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="F51" s="3"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="4" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="B52" s="5"/>
       <c r="C52" s="5"/>
@@ -1824,7 +2361,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B53" s="7">
         <v>78.853999999999999</v>
@@ -1841,7 +2378,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="6" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B54" s="7">
         <v>82.819000000000003</v>
@@ -1858,7 +2395,7 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="6" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B55" s="7">
         <v>105.15600000000001</v>
@@ -1875,7 +2412,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="6" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B56" s="7">
         <v>150.10499999999999</v>
@@ -1892,7 +2429,7 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B57" s="7">
         <v>60.484000000000002</v>
@@ -1909,7 +2446,7 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="4" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="B58" s="5"/>
       <c r="C58" s="5"/>
@@ -1919,7 +2456,7 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="9" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B59" s="10">
         <v>46.009</v>
@@ -1936,7 +2473,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="9" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B60" s="10">
         <v>57.712000000000003</v>
@@ -1953,7 +2490,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="9" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B61" s="10">
         <v>60.438000000000002</v>
@@ -1970,7 +2507,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="9" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B62" s="10">
         <v>60.616999999999997</v>
@@ -1987,7 +2524,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="9" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B63" s="10">
         <v>40.393000000000001</v>
@@ -2004,30 +2541,30 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="32" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="33" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="B66" s="33" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C66" s="33" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="D66" s="33" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E66" s="33" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="F66" s="33"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="34" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="B67" s="35"/>
       <c r="C67" s="35"/>
@@ -2037,7 +2574,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="36" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B68" s="37">
         <v>86.75</v>
@@ -2054,7 +2591,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="36" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B69" s="37">
         <v>92.5</v>
@@ -2071,7 +2608,7 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="36" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B70" s="37">
         <v>114.896</v>
@@ -2088,7 +2625,7 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="36" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B71" s="37">
         <v>166.76400000000001</v>
@@ -2105,7 +2642,7 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="36" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B72" s="37">
         <v>63.59</v>
@@ -2122,7 +2659,7 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="34" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="B73" s="35"/>
       <c r="C73" s="35"/>
@@ -2132,7 +2669,7 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="36" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B74" s="37">
         <v>37.722000000000001</v>
@@ -2149,7 +2686,7 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="36" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B75" s="37">
         <v>61.936999999999998</v>
@@ -2166,7 +2703,7 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="36" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B76" s="37">
         <v>86.201999999999998</v>
@@ -2183,7 +2720,7 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="36" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B77" s="37">
         <v>137.834</v>
@@ -2200,7 +2737,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="36" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B78" s="37">
         <v>74.051000000000002</v>
@@ -2217,7 +2754,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" s="34" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -2227,7 +2764,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="39" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B80" s="40">
         <v>30.827999999999999</v>
@@ -2244,7 +2781,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" s="39" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B81" s="40">
         <v>57.758000000000003</v>
@@ -2261,7 +2798,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="39" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B82" s="40">
         <v>80.587999999999994</v>
@@ -2278,7 +2815,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" s="39" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B83" s="40">
         <v>132.24799999999999</v>
@@ -2295,7 +2832,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="39" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B84" s="40">
         <v>64.989999999999995</v>
@@ -2311,41 +2848,41 @@
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A86" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="B86" s="43"/>
-      <c r="C86" s="43"/>
-      <c r="D86" s="43"/>
-      <c r="E86" s="43"/>
-      <c r="F86" s="43"/>
+      <c r="A86" s="53" t="s">
+        <v>56</v>
+      </c>
+      <c r="B86" s="52"/>
+      <c r="C86" s="52"/>
+      <c r="D86" s="52"/>
+      <c r="E86" s="52"/>
+      <c r="F86" s="52"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" s="32" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" s="33" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="B89" s="33" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C89" s="33" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="D89" s="33" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E89" s="33" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="F89" s="33"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" s="34" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="B90" s="35"/>
       <c r="C90" s="35"/>
@@ -2355,7 +2892,7 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" s="36" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B91" s="37">
         <v>66.841999999999999</v>
@@ -2372,7 +2909,7 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" s="36" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B92" s="37">
         <v>66.947000000000003</v>
@@ -2389,7 +2926,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" s="36" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B93" s="37">
         <v>68.572999999999993</v>
@@ -2406,7 +2943,7 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" s="36" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B94" s="37">
         <v>66.213999999999999</v>
@@ -2423,7 +2960,7 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" s="34" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B95" s="35"/>
       <c r="C95" s="35"/>
@@ -2433,7 +2970,7 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" s="36" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B96" s="37">
         <v>60.097000000000001</v>
@@ -2450,7 +2987,7 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" s="36" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B97" s="37">
         <v>70.33</v>
@@ -2467,7 +3004,7 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" s="36" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B98" s="37">
         <v>68.334999999999994</v>
@@ -2484,7 +3021,7 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" s="36" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B99" s="37">
         <v>64.048000000000002</v>
@@ -2501,7 +3038,7 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" s="34" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B100" s="35"/>
       <c r="C100" s="35"/>
@@ -2511,7 +3048,7 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" s="39" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B101" s="40">
         <v>33.468000000000004</v>
@@ -2528,7 +3065,7 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" s="39" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B102" s="40">
         <v>49.607999999999997</v>
@@ -2545,7 +3082,7 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" s="39" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B103" s="40">
         <v>60.097999999999999</v>
@@ -2562,7 +3099,7 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" s="39" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B104" s="40">
         <v>65.522999999999996</v>
@@ -2578,14 +3115,14 @@
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A106" s="45" t="s">
-        <v>31</v>
-      </c>
-      <c r="B106" s="43"/>
-      <c r="C106" s="43"/>
-      <c r="D106" s="43"/>
-      <c r="E106" s="43"/>
-      <c r="F106" s="43"/>
+      <c r="A106" s="53" t="s">
+        <v>58</v>
+      </c>
+      <c r="B106" s="52"/>
+      <c r="C106" s="52"/>
+      <c r="D106" s="52"/>
+      <c r="E106" s="52"/>
+      <c r="F106" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2600,8 +3137,845 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:F63"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="36" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="55" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="49" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="32" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" s="33"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="35"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="37">
+        <v>24.59</v>
+      </c>
+      <c r="C8" s="37">
+        <v>40.237000000000002</v>
+      </c>
+      <c r="D8" s="38">
+        <v>0.41499999999999998</v>
+      </c>
+      <c r="E8" s="37">
+        <v>69.323999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="37">
+        <v>36.384</v>
+      </c>
+      <c r="C9" s="37">
+        <v>57.58</v>
+      </c>
+      <c r="D9" s="38">
+        <v>0.61399999999999999</v>
+      </c>
+      <c r="E9" s="37">
+        <v>119.887</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="37">
+        <v>49.203000000000003</v>
+      </c>
+      <c r="C10" s="37">
+        <v>77.472999999999999</v>
+      </c>
+      <c r="D10" s="38">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="E10" s="37">
+        <v>154.768</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="43" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="37">
+        <v>56.314</v>
+      </c>
+      <c r="C11" s="37">
+        <v>86.875</v>
+      </c>
+      <c r="D11" s="38">
+        <v>0.95099999999999996</v>
+      </c>
+      <c r="E11" s="37">
+        <v>192.99199999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="44">
+        <v>27.608000000000001</v>
+      </c>
+      <c r="C13" s="44">
+        <v>41.631</v>
+      </c>
+      <c r="D13" s="45">
+        <v>0.46100000000000002</v>
+      </c>
+      <c r="E13" s="44">
+        <v>66.804000000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="44">
+        <v>28.975000000000001</v>
+      </c>
+      <c r="C14" s="44">
+        <v>44.469000000000001</v>
+      </c>
+      <c r="D14" s="45">
+        <v>0.48299999999999998</v>
+      </c>
+      <c r="E14" s="44">
+        <v>66.671999999999997</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="44">
+        <v>33.085000000000001</v>
+      </c>
+      <c r="C15" s="44">
+        <v>54.441000000000003</v>
+      </c>
+      <c r="D15" s="45">
+        <v>0.55200000000000005</v>
+      </c>
+      <c r="E15" s="44">
+        <v>71.070999999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="44">
+        <v>34.085999999999999</v>
+      </c>
+      <c r="C16" s="44">
+        <v>54.17</v>
+      </c>
+      <c r="D16" s="45">
+        <v>0.56899999999999995</v>
+      </c>
+      <c r="E16" s="44">
+        <v>75.820999999999998</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="32" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" s="33"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="37">
+        <v>22.87</v>
+      </c>
+      <c r="C21" s="37">
+        <v>39.375</v>
+      </c>
+      <c r="D21" s="38">
+        <v>0.38900000000000001</v>
+      </c>
+      <c r="E21" s="37">
+        <v>83.073999999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="37">
+        <v>36.186999999999998</v>
+      </c>
+      <c r="C22" s="37">
+        <v>58.905000000000001</v>
+      </c>
+      <c r="D22" s="38">
+        <v>0.61699999999999999</v>
+      </c>
+      <c r="E22" s="37">
+        <v>131.297</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="B23" s="37">
+        <v>48.31</v>
+      </c>
+      <c r="C23" s="37">
+        <v>77.585999999999999</v>
+      </c>
+      <c r="D23" s="38">
+        <v>0.82399999999999995</v>
+      </c>
+      <c r="E23" s="37">
+        <v>172.71700000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="43" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="37">
+        <v>52.207999999999998</v>
+      </c>
+      <c r="C24" s="37">
+        <v>79.683999999999997</v>
+      </c>
+      <c r="D24" s="38">
+        <v>0.89100000000000001</v>
+      </c>
+      <c r="E24" s="37">
+        <v>199.61600000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="35"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="44">
+        <v>26.209</v>
+      </c>
+      <c r="C26" s="44">
+        <v>41.338999999999999</v>
+      </c>
+      <c r="D26" s="45">
+        <v>0.44400000000000001</v>
+      </c>
+      <c r="E26" s="44">
+        <v>65.527000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="44">
+        <v>28.187999999999999</v>
+      </c>
+      <c r="C27" s="44">
+        <v>45.524999999999999</v>
+      </c>
+      <c r="D27" s="45">
+        <v>0.48</v>
+      </c>
+      <c r="E27" s="44">
+        <v>68.253</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" s="44">
+        <v>33.006</v>
+      </c>
+      <c r="C28" s="44">
+        <v>56.713000000000001</v>
+      </c>
+      <c r="D28" s="45">
+        <v>0.56200000000000006</v>
+      </c>
+      <c r="E28" s="44">
+        <v>72.512</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" s="44">
+        <v>34.847000000000001</v>
+      </c>
+      <c r="C29" s="44">
+        <v>58.186999999999998</v>
+      </c>
+      <c r="D29" s="45">
+        <v>0.59399999999999997</v>
+      </c>
+      <c r="E29" s="44">
+        <v>79.620999999999995</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="49" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="32" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="D33" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="E33" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="F33" s="33"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="B34" s="35"/>
+      <c r="C34" s="35"/>
+      <c r="D34" s="35"/>
+      <c r="E34" s="35"/>
+      <c r="F34" s="35"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="37">
+        <v>29.381</v>
+      </c>
+      <c r="C35" s="37">
+        <v>51.131</v>
+      </c>
+      <c r="D35" s="38">
+        <v>0.49</v>
+      </c>
+      <c r="E35" s="37">
+        <v>76.301000000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="37">
+        <v>41.018000000000001</v>
+      </c>
+      <c r="C36" s="37">
+        <v>66.722999999999999</v>
+      </c>
+      <c r="D36" s="38">
+        <v>0.68400000000000005</v>
+      </c>
+      <c r="E36" s="37">
+        <v>133.29</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="37">
+        <v>54.070999999999998</v>
+      </c>
+      <c r="C37" s="37">
+        <v>85.4</v>
+      </c>
+      <c r="D37" s="38">
+        <v>0.90200000000000002</v>
+      </c>
+      <c r="E37" s="37">
+        <v>169.547</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="43" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="37">
+        <v>59.186</v>
+      </c>
+      <c r="C38" s="37">
+        <v>89.575999999999993</v>
+      </c>
+      <c r="D38" s="38">
+        <v>0.98799999999999999</v>
+      </c>
+      <c r="E38" s="37">
+        <v>201.50700000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B39" s="35"/>
+      <c r="C39" s="35"/>
+      <c r="D39" s="35"/>
+      <c r="E39" s="35"/>
+      <c r="F39" s="35"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B40" s="44">
+        <v>29.321999999999999</v>
+      </c>
+      <c r="C40" s="44">
+        <v>49.399000000000001</v>
+      </c>
+      <c r="D40" s="45">
+        <v>0.48899999999999999</v>
+      </c>
+      <c r="E40" s="44">
+        <v>86.94</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B41" s="44">
+        <v>39.579000000000001</v>
+      </c>
+      <c r="C41" s="44">
+        <v>64.721000000000004</v>
+      </c>
+      <c r="D41" s="45">
+        <v>0.66</v>
+      </c>
+      <c r="E41" s="44">
+        <v>132.21</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="B42" s="44">
+        <v>52.52</v>
+      </c>
+      <c r="C42" s="44">
+        <v>84.59</v>
+      </c>
+      <c r="D42" s="45">
+        <v>0.876</v>
+      </c>
+      <c r="E42" s="44">
+        <v>156.31399999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="B43" s="44">
+        <v>56.28</v>
+      </c>
+      <c r="C43" s="44">
+        <v>86.962999999999994</v>
+      </c>
+      <c r="D43" s="45">
+        <v>0.93899999999999995</v>
+      </c>
+      <c r="E43" s="44">
+        <v>171.99799999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" s="32" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="B46" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C46" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="D46" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="E46" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="F46" s="33"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B47" s="35"/>
+      <c r="C47" s="35"/>
+      <c r="D47" s="35"/>
+      <c r="E47" s="35"/>
+      <c r="F47" s="35"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B48" s="44">
+        <v>29.361000000000001</v>
+      </c>
+      <c r="C48" s="44">
+        <v>48.107999999999997</v>
+      </c>
+      <c r="D48" s="45">
+        <v>0.498</v>
+      </c>
+      <c r="E48" s="44">
+        <v>78.930000000000007</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B49" s="44">
+        <v>39.758000000000003</v>
+      </c>
+      <c r="C49" s="44">
+        <v>64.606999999999999</v>
+      </c>
+      <c r="D49" s="45">
+        <v>0.67700000000000005</v>
+      </c>
+      <c r="E49" s="44">
+        <v>144.27099999999999</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A50" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="B50" s="44">
+        <v>51.216999999999999</v>
+      </c>
+      <c r="C50" s="44">
+        <v>82.162999999999997</v>
+      </c>
+      <c r="D50" s="45">
+        <v>0.872</v>
+      </c>
+      <c r="E50" s="44">
+        <v>186.72</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A51" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="B51" s="44">
+        <v>55.454999999999998</v>
+      </c>
+      <c r="C51" s="44">
+        <v>85.441999999999993</v>
+      </c>
+      <c r="D51" s="45">
+        <v>0.94499999999999995</v>
+      </c>
+      <c r="E51" s="44">
+        <v>214.54900000000001</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A52" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="B52" s="35"/>
+      <c r="C52" s="35"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="35"/>
+      <c r="F52" s="35"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A53" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="B53" s="37">
+        <v>29.657</v>
+      </c>
+      <c r="C53" s="37">
+        <v>50.088000000000001</v>
+      </c>
+      <c r="D53" s="38">
+        <v>0.503</v>
+      </c>
+      <c r="E53" s="37">
+        <v>91.844999999999999</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A54" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="B54" s="37">
+        <v>41.271999999999998</v>
+      </c>
+      <c r="C54" s="37">
+        <v>67.471999999999994</v>
+      </c>
+      <c r="D54" s="38">
+        <v>0.70199999999999996</v>
+      </c>
+      <c r="E54" s="37">
+        <v>128.108</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A55" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="B55" s="37">
+        <v>53.71</v>
+      </c>
+      <c r="C55" s="37">
+        <v>88.049000000000007</v>
+      </c>
+      <c r="D55" s="38">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="E55" s="37">
+        <v>147.99100000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A56" s="43" t="s">
+        <v>40</v>
+      </c>
+      <c r="B56" s="37">
+        <v>59.103999999999999</v>
+      </c>
+      <c r="C56" s="37">
+        <v>92.503</v>
+      </c>
+      <c r="D56" s="38">
+        <v>1.006</v>
+      </c>
+      <c r="E56" s="37">
+        <v>178.00399999999999</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A58" s="46" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="46" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="B59" s="59" t="s">
+        <v>74</v>
+      </c>
+      <c r="C59" s="52"/>
+      <c r="D59" s="52"/>
+      <c r="E59" s="52"/>
+      <c r="F59" s="52"/>
+    </row>
+    <row r="60" spans="1:6" ht="46" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="47" t="s">
+        <v>75</v>
+      </c>
+      <c r="B60" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C60" s="52"/>
+      <c r="D60" s="52"/>
+      <c r="E60" s="52"/>
+      <c r="F60" s="52"/>
+    </row>
+    <row r="61" spans="1:6" ht="46" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="47" t="s">
+        <v>77</v>
+      </c>
+      <c r="B61" s="59" t="s">
+        <v>78</v>
+      </c>
+      <c r="C61" s="52"/>
+      <c r="D61" s="52"/>
+      <c r="E61" s="52"/>
+      <c r="F61" s="52"/>
+    </row>
+    <row r="62" spans="1:6" ht="46" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="47" t="s">
+        <v>79</v>
+      </c>
+      <c r="B62" s="59" t="s">
+        <v>80</v>
+      </c>
+      <c r="C62" s="52"/>
+      <c r="D62" s="52"/>
+      <c r="E62" s="52"/>
+      <c r="F62" s="52"/>
+    </row>
+    <row r="63" spans="1:6" ht="46" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A63" s="47" t="s">
+        <v>81</v>
+      </c>
+      <c r="B63" s="59" t="s">
+        <v>82</v>
+      </c>
+      <c r="C63" s="52"/>
+      <c r="D63" s="52"/>
+      <c r="E63" s="52"/>
+      <c r="F63" s="52"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="B61:F61"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B62:F62"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B59:F59"/>
+    <mergeCell ref="B60:F60"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2616,72 +3990,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
+      <c r="A1" s="56" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="46" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
+      <c r="A2" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>37</v>
+        <v>87</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>38</v>
+        <v>88</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>41</v>
+        <v>91</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="J4" s="30" t="s">
-        <v>43</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="15" t="s">
-        <v>44</v>
+        <v>94</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="D5" s="16">
         <v>50.1</v>
@@ -2690,30 +4064,30 @@
         <v>37.6</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="G5" s="17">
         <v>2026</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>49</v>
+        <v>99</v>
       </c>
       <c r="J5" s="31" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
-        <v>51</v>
+        <v>101</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="D6" s="16">
         <v>50.08</v>
@@ -2722,30 +4096,30 @@
         <v>37.67</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="G6" s="17">
         <v>2026</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="J6" s="31" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
-        <v>53</v>
+        <v>103</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="D7" s="16">
         <v>46.85</v>
@@ -2754,30 +4128,30 @@
         <v>32.5</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="G7" s="17">
         <v>2026</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>55</v>
+        <v>105</v>
       </c>
       <c r="J7" s="31" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
-        <v>56</v>
+        <v>106</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>57</v>
+        <v>107</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="D8" s="16">
         <v>228.87</v>
@@ -2786,30 +4160,30 @@
         <v>140.55000000000001</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="G8" s="17">
         <v>2026</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>58</v>
+        <v>108</v>
       </c>
       <c r="J8" s="31" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="12" t="s">
-        <v>59</v>
+        <v>109</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>61</v>
+        <v>111</v>
       </c>
       <c r="D9" s="13">
         <v>8.81</v>
@@ -2818,59 +4192,59 @@
         <v>5.04</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="G9" s="18">
         <v>2025</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>62</v>
+        <v>112</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>63</v>
+        <v>113</v>
       </c>
       <c r="J9" s="31" t="s">
-        <v>64</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>65</v>
+        <v>115</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>66</v>
+        <v>116</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
       <c r="D10" s="7">
         <v>82</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="G10" s="19">
         <v>2026</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>69</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>66</v>
+        <v>116</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
       <c r="D11" s="7">
         <v>19.899999999999999</v>
@@ -2885,27 +4259,27 @@
         <v>2026</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>71</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>72</v>
+        <v>122</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>73</v>
+        <v>123</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
       <c r="D12" s="7">
         <v>15.6</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="F12" s="8">
         <v>0.96399999999999997</v>
@@ -2914,27 +4288,27 @@
         <v>2026</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>74</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>75</v>
+        <v>125</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
       <c r="D13" s="7">
         <v>13.7</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="F13" s="8">
         <v>0.97199999999999998</v>
@@ -2943,21 +4317,21 @@
         <v>2026</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>77</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>78</v>
+        <v>128</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
       <c r="D14" s="7">
         <v>26.6</v>
@@ -2972,27 +4346,27 @@
         <v>2026</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>79</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>73</v>
+        <v>123</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
       <c r="D15" s="7">
         <v>65.7</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="F15" s="8">
         <v>0.379</v>
@@ -3001,21 +4375,21 @@
         <v>2026</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
-        <v>82</v>
+        <v>132</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>83</v>
+        <v>133</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>84</v>
+        <v>134</v>
       </c>
       <c r="D16" s="7">
         <v>19</v>
@@ -3030,21 +4404,21 @@
         <v>2023</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>85</v>
+        <v>135</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>86</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="53" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
-        <v>87</v>
+        <v>137</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>88</v>
+        <v>138</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>89</v>
+        <v>139</v>
       </c>
       <c r="D17" s="16">
         <v>18.899999999999999</v>
@@ -3059,24 +4433,24 @@
         <v>2022</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>91</v>
+        <v>141</v>
       </c>
       <c r="J17" s="31" t="s">
-        <v>92</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
-        <v>93</v>
+        <v>143</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>88</v>
+        <v>138</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>94</v>
+        <v>144</v>
       </c>
       <c r="D18" s="7">
         <v>12.9</v>
@@ -3085,110 +4459,110 @@
         <v>6.7</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="G18" s="19">
         <v>2020</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>96</v>
+        <v>146</v>
       </c>
       <c r="J18" s="31" t="s">
-        <v>97</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>98</v>
+        <v>148</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>99</v>
+        <v>149</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="G19" s="19">
         <v>2025</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>101</v>
+        <v>151</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>102</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="20" t="s">
-        <v>103</v>
+        <v>153</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>104</v>
+        <v>154</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>105</v>
+        <v>155</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="E20" s="21" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="F20" s="21" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="G20" s="21">
         <v>2017</v>
       </c>
       <c r="H20" s="20" t="s">
-        <v>106</v>
+        <v>156</v>
       </c>
       <c r="I20" s="20" t="s">
-        <v>107</v>
+        <v>157</v>
       </c>
       <c r="J20" s="31" t="s">
-        <v>108</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="J21" s="31" t="s">
-        <v>109</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I20" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A4:I20" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="J5" r:id="rId1" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Interpretabel PM25 Forecasting_2026.pdf" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="J6" r:id="rId2" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Interpretabel PM25 Forecasting_2026.pdf" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="J7" r:id="rId3" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Interpretabel PM25 Forecasting_2026.pdf" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="J8" r:id="rId4" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Interpretabel PM25 Forecasting_2026.pdf" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
-    <hyperlink ref="J9" r:id="rId5" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Designing a residual-enhanced_2025.pdf" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
-    <hyperlink ref="J17" r:id="rId6" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Prediction_of_Multi-Site_PM25_Concentrations_in_Be.pdf" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
-    <hyperlink ref="J18" r:id="rId7" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Multi hour and multi site abstract 2022.pdf" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
-    <hyperlink ref="J20" r:id="rId8" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/rspa.2017.0457.pdf" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
-    <hyperlink ref="J21" r:id="rId9" display="https://github.com/dolcikey/TimeSeriesForecasting_BeijingAirQuality" xr:uid="{00000000-0004-0000-0100-000008000000}"/>
+    <hyperlink ref="J5" r:id="rId1" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Interpretabel PM25 Forecasting_2026.pdf" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="J6" r:id="rId2" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Interpretabel PM25 Forecasting_2026.pdf" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="J7" r:id="rId3" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Interpretabel PM25 Forecasting_2026.pdf" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
+    <hyperlink ref="J8" r:id="rId4" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Interpretabel PM25 Forecasting_2026.pdf" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
+    <hyperlink ref="J9" r:id="rId5" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Designing a residual-enhanced_2025.pdf" xr:uid="{00000000-0004-0000-0300-000004000000}"/>
+    <hyperlink ref="J17" r:id="rId6" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Prediction_of_Multi-Site_PM25_Concentrations_in_Be.pdf" xr:uid="{00000000-0004-0000-0300-000005000000}"/>
+    <hyperlink ref="J18" r:id="rId7" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/Multi hour and multi site abstract 2022.pdf" xr:uid="{00000000-0004-0000-0300-000006000000}"/>
+    <hyperlink ref="J20" r:id="rId8" display="https://github.com/KaiSteffen/Business-Prognosis/blob/main/Capstone Projekt/literature/rspa.2017.0457.pdf" xr:uid="{00000000-0004-0000-0300-000007000000}"/>
+    <hyperlink ref="J21" r:id="rId9" display="https://github.com/dolcikey/TimeSeriesForecasting_BeijingAirQuality" xr:uid="{00000000-0004-0000-0300-000008000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3198,82 +4572,82 @@
   <sheetData>
     <row r="1" spans="2:2" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B1" s="22" t="s">
-        <v>110</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B2" s="23" t="s">
-        <v>111</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B4" s="2" t="s">
-        <v>112</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="2:2" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="24" t="s">
-        <v>113</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B7" s="2" t="s">
-        <v>114</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="2:2" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="24" t="s">
-        <v>115</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B10" s="2" t="s">
-        <v>116</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="2:2" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="24" t="s">
-        <v>117</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B13" s="2" t="s">
-        <v>118</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="2:2" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="24" t="s">
-        <v>119</v>
+        <v>169</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B16" s="2" t="s">
-        <v>120</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="2:2" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="24" t="s">
-        <v>121</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" s="2" t="s">
-        <v>122</v>
+        <v>172</v>
       </c>
     </row>
     <row r="20" spans="2:2" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="24" t="s">
-        <v>123</v>
+        <v>173</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B22" s="2" t="s">
-        <v>124</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23" spans="2:2" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="24" t="s">
-        <v>125</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -3281,8 +4655,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B1:C19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3292,96 +4666,96 @@
   <sheetData>
     <row r="1" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B1" s="1" t="s">
-        <v>126</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
-        <v>127</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="2:3" ht="64" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="24" t="s">
-        <v>128</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
-        <v>129</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="64" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="24" t="s">
-        <v>130</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B9" s="2" t="s">
-        <v>131</v>
+        <v>181</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>132</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="64" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="24" t="s">
-        <v>133</v>
+        <v>183</v>
       </c>
       <c r="C10" s="27"/>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C11" s="28" t="s">
-        <v>134</v>
+        <v>184</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B12" s="2" t="s">
-        <v>135</v>
+        <v>185</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>136</v>
+        <v>186</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="64" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="24" t="s">
-        <v>137</v>
+        <v>187</v>
       </c>
       <c r="C13" s="28" t="s">
-        <v>138</v>
+        <v>188</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C14" s="28" t="s">
-        <v>139</v>
+        <v>189</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B15" s="2" t="s">
-        <v>140</v>
+        <v>190</v>
       </c>
       <c r="C15" s="28" t="s">
-        <v>141</v>
+        <v>191</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="64" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="24" t="s">
-        <v>142</v>
+        <v>192</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>143</v>
+        <v>193</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B18" s="2" t="s">
-        <v>144</v>
+        <v>194</v>
       </c>
       <c r="C18" t="s">
-        <v>145</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="64" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="24" t="s">
-        <v>146</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -3389,8 +4763,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="B1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3401,82 +4775,82 @@
   <sheetData>
     <row r="1" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B1" s="25" t="s">
-        <v>41</v>
+        <v>91</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>147</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="24" t="s">
-        <v>148</v>
+        <v>198</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>149</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="24" t="s">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>151</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="24" t="s">
-        <v>152</v>
+        <v>202</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>153</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="24" t="s">
-        <v>154</v>
+        <v>204</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>155</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="24" t="s">
-        <v>156</v>
+        <v>206</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="24" t="s">
-        <v>157</v>
+        <v>207</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>158</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="24" t="s">
-        <v>159</v>
+        <v>209</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>160</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="24" t="s">
-        <v>161</v>
+        <v>211</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>162</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="24" t="s">
-        <v>164</v>
+        <v>213</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>163</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>